<commit_message>
Deploying to gh-pages from  @ 92a757512d4f3051c0aaf89352db4feb6d0964e6 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_5-1-1.xlsx
+++ b/assets/excel/2026_5-1-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99E33C8-FD71-4DF0-A99A-311440119DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC2884A8-9516-4A5E-9258-FBA01E98AFCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{FAA839E9-FEB0-4C88-9D08-E3A9182EBE0D}"/>
+    <workbookView xWindow="20052" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FAA839E9-FEB0-4C88-9D08-E3A9182EBE0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="2" r:id="rId1"/>
@@ -135,12 +135,6 @@
     <t>/</t>
   </si>
   <si>
-    <t>1) Die Angabe des Wirtschaftszweiges erfolgte ab Erhebungsjahr 2009 nach der Klassifikation der Wirtschaftszweige, Ausgabe 2008 (WZ 2008). Im Jahr 2005 wurde hingegen die zu diesem Zeitpunkt gültige Klassifikation der Wirtschaftszweige, Ausgabe 2003 (WZ 2003), zugrunde gelegt. Aufgrund von größeren Verschiebungen bzw. Änderungen in den fachlichen Zuordnungen sind die dargestellten Werte des Erhebungsjahres 2005 und ab den Jahren 2009 nur sehr eingeschränkt vergleichbar.</t>
-  </si>
-  <si>
-    <t>3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020, 2021 und 2022 finden Sie auf der Informationsseite des Statistischen Bundesamtes</t>
-  </si>
-  <si>
     <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Haushalte-Familien/Methoden/mikrozensus-2020.html</t>
   </si>
   <si>
@@ -162,10 +156,16 @@
     <t>Jahr2)</t>
   </si>
   <si>
-    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,                                                   </t>
+    <t>2) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
   </si>
   <si>
-    <t>2) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
+    <t>1)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren.</t>
+  </si>
+  <si>
+    <t>3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes:</t>
+  </si>
+  <si>
+    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,</t>
   </si>
 </sst>
 </file>
@@ -500,12 +500,6 @@
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -517,6 +511,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -556,11 +556,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -583,9 +583,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -623,7 +623,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -729,7 +729,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -871,7 +871,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -880,7 +880,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3A0A6A-188A-48ED-893A-2E9C55642D8A}">
   <sheetPr codeName="Tabelle2"/>
-  <dimension ref="B1:I187"/>
+  <dimension ref="B1:M187"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
@@ -888,8 +888,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="46" t="s">
-        <v>32</v>
+      <c r="B1" s="31" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -897,15 +897,15 @@
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
     </row>
     <row r="4" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="47" t="s">
+      <c r="B4" s="32" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="2"/>
@@ -920,7 +920,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D6" s="39" t="s">
         <v>3</v>
@@ -3781,99 +3781,194 @@
       </c>
     </row>
     <row r="176" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B176" s="28"/>
-    </row>
-    <row r="177" spans="2:9" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B177" s="27" t="s">
+      <c r="B176" s="26"/>
+    </row>
+    <row r="177" spans="2:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B177" s="46" t="s">
+        <v>33</v>
+      </c>
+      <c r="C177" s="46"/>
+      <c r="D177" s="46"/>
+      <c r="E177" s="46"/>
+      <c r="F177" s="46"/>
+      <c r="G177" s="46"/>
+      <c r="H177" s="46"/>
+      <c r="I177" s="46"/>
+      <c r="J177" s="46"/>
+      <c r="K177" s="46"/>
+      <c r="L177" s="46"/>
+      <c r="M177" s="46"/>
+    </row>
+    <row r="178" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B178" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="C178" s="46"/>
+      <c r="D178" s="46"/>
+      <c r="E178" s="46"/>
+      <c r="F178" s="46"/>
+      <c r="G178" s="46"/>
+      <c r="H178" s="46"/>
+      <c r="I178" s="46"/>
+      <c r="J178" s="46"/>
+      <c r="K178" s="46"/>
+      <c r="L178" s="46"/>
+      <c r="M178" s="46"/>
+    </row>
+    <row r="179" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B179" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="C179" s="46"/>
+      <c r="D179" s="46"/>
+      <c r="E179" s="46"/>
+      <c r="F179" s="46"/>
+      <c r="G179" s="46"/>
+      <c r="H179" s="46"/>
+      <c r="I179" s="46"/>
+      <c r="J179" s="46"/>
+      <c r="K179" s="46"/>
+      <c r="L179" s="46"/>
+      <c r="M179" s="46"/>
+    </row>
+    <row r="180" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B180" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C177" s="27"/>
-      <c r="D177" s="27"/>
-      <c r="E177" s="27"/>
-      <c r="F177" s="27"/>
-      <c r="G177" s="27"/>
-      <c r="H177" s="27"/>
-      <c r="I177" s="27"/>
-    </row>
-    <row r="178" spans="2:9" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B178" s="27" t="s">
+      <c r="C180" s="47"/>
+      <c r="D180" s="47"/>
+      <c r="E180" s="47"/>
+      <c r="F180" s="47"/>
+      <c r="G180" s="47"/>
+      <c r="H180" s="47"/>
+      <c r="I180" s="47"/>
+      <c r="J180" s="47"/>
+      <c r="K180" s="47"/>
+      <c r="L180" s="47"/>
+      <c r="M180" s="47"/>
+    </row>
+    <row r="181" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B181" s="27"/>
+      <c r="C181" s="47"/>
+      <c r="D181" s="47"/>
+      <c r="E181" s="47"/>
+      <c r="F181" s="47"/>
+      <c r="G181" s="47"/>
+      <c r="H181" s="47"/>
+      <c r="I181" s="47"/>
+      <c r="J181" s="47"/>
+      <c r="K181" s="47"/>
+      <c r="L181" s="47"/>
+      <c r="M181" s="47"/>
+    </row>
+    <row r="182" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B182" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C182" s="47"/>
+      <c r="D182" s="47"/>
+      <c r="E182" s="47"/>
+      <c r="F182" s="47"/>
+      <c r="G182" s="47"/>
+      <c r="H182" s="47"/>
+      <c r="I182" s="47"/>
+      <c r="J182" s="47"/>
+      <c r="K182" s="47"/>
+      <c r="L182" s="47"/>
+      <c r="M182" s="47"/>
+    </row>
+    <row r="183" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B183" s="47"/>
+      <c r="C183" s="47"/>
+      <c r="D183" s="47"/>
+      <c r="E183" s="47"/>
+      <c r="F183" s="47"/>
+      <c r="G183" s="47"/>
+      <c r="H183" s="47"/>
+      <c r="I183" s="47"/>
+      <c r="J183" s="47"/>
+      <c r="K183" s="47"/>
+      <c r="L183" s="47"/>
+      <c r="M183" s="47"/>
+    </row>
+    <row r="184" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B184" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C184" s="47"/>
+      <c r="D184" s="47"/>
+      <c r="E184" s="47"/>
+      <c r="F184" s="47"/>
+      <c r="G184" s="47"/>
+      <c r="H184" s="47"/>
+      <c r="I184" s="47"/>
+      <c r="J184" s="47"/>
+      <c r="K184" s="47"/>
+      <c r="L184" s="47"/>
+      <c r="M184" s="47"/>
+    </row>
+    <row r="185" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B185" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="C178" s="27"/>
-      <c r="D178" s="27"/>
-      <c r="E178" s="27"/>
-      <c r="F178" s="27"/>
-      <c r="G178" s="27"/>
-      <c r="H178" s="27"/>
-      <c r="I178" s="27"/>
-    </row>
-    <row r="179" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B179" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="C179" s="27"/>
-      <c r="D179" s="27"/>
-      <c r="E179" s="27"/>
-      <c r="F179" s="27"/>
-      <c r="G179" s="27"/>
-      <c r="H179" s="27"/>
-      <c r="I179" s="27"/>
-    </row>
-    <row r="180" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B180" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="C180" s="26"/>
-      <c r="D180" s="26"/>
-      <c r="E180" s="26"/>
-      <c r="F180" s="26"/>
-      <c r="G180" s="26"/>
-      <c r="H180" s="26"/>
-      <c r="I180" s="26"/>
-    </row>
-    <row r="181" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B181" s="29"/>
-      <c r="C181" s="26"/>
-      <c r="D181" s="26"/>
-      <c r="E181" s="26"/>
-      <c r="F181" s="26"/>
-      <c r="G181" s="26"/>
-      <c r="H181" s="26"/>
-      <c r="I181" s="26"/>
-    </row>
-    <row r="182" spans="2:9" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B182" s="25" t="s">
+      <c r="C185" s="47"/>
+      <c r="D185" s="47"/>
+      <c r="E185" s="47"/>
+      <c r="F185" s="47"/>
+      <c r="G185" s="47"/>
+      <c r="H185" s="47"/>
+      <c r="I185" s="47"/>
+      <c r="J185" s="47"/>
+      <c r="K185" s="47"/>
+      <c r="L185" s="47"/>
+      <c r="M185" s="47"/>
+    </row>
+    <row r="186" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B186" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C182" s="25"/>
-    </row>
-    <row r="184" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B184" s="30" t="s">
+      <c r="C186" s="47"/>
+      <c r="D186" s="47"/>
+      <c r="E186" s="47"/>
+      <c r="F186" s="47"/>
+      <c r="G186" s="47"/>
+      <c r="H186" s="47"/>
+      <c r="I186" s="47"/>
+      <c r="J186" s="47"/>
+      <c r="K186" s="47"/>
+      <c r="L186" s="47"/>
+      <c r="M186" s="47"/>
+    </row>
+    <row r="187" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B187" s="29" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="185" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B185" s="30" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="186" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B186" s="30" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="187" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B187" s="31" t="s">
-        <v>31</v>
-      </c>
+      <c r="C187" s="47"/>
+      <c r="D187" s="47"/>
+      <c r="E187" s="47"/>
+      <c r="F187" s="47"/>
+      <c r="G187" s="47"/>
+      <c r="H187" s="47"/>
+      <c r="I187" s="47"/>
+      <c r="J187" s="47"/>
+      <c r="K187" s="47"/>
+      <c r="L187" s="47"/>
+      <c r="M187" s="47"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
+    <mergeCell ref="B178:M178"/>
+    <mergeCell ref="B179:M179"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="C6:C9"/>
     <mergeCell ref="D6:F7"/>
     <mergeCell ref="D9:F9"/>
+    <mergeCell ref="B177:M177"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B180" r:id="rId1" xr:uid="{14A69F6D-C1C7-4DC1-9F40-1C9E12EA0EFC}"/>
+    <hyperlink ref="B187" r:id="rId2" xr:uid="{4A998CE4-8818-461C-8C35-B06AC0C8039B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>